<commit_message>
Template prospect nettoyé + doc synchronisation + routes download
</commit_message>
<xml_diff>
--- a/templates/TEMPLATE_FICHE_PROSPECT.xlsx
+++ b/templates/TEMPLATE_FICHE_PROSPECT.xlsx
@@ -1177,7 +1177,7 @@
       </c>
       <c r="E4" s="81" t="inlineStr">
         <is>
-          <t>Évaluation</t>
+          <t>❓</t>
         </is>
       </c>
     </row>
@@ -1195,7 +1195,7 @@
       </c>
       <c r="E5" s="85" t="inlineStr">
         <is>
-          <t>✅ Très solide</t>
+          <t>❓</t>
         </is>
       </c>
     </row>
@@ -1213,7 +1213,7 @@
       </c>
       <c r="E6" s="85" t="inlineStr">
         <is>
-          <t>✅ Partenaire historique</t>
+          <t>❓</t>
         </is>
       </c>
     </row>
@@ -1231,7 +1231,7 @@
       </c>
       <c r="E7" s="85" t="inlineStr">
         <is>
-          <t>✅ Dossier complet</t>
+          <t>❓</t>
         </is>
       </c>
     </row>
@@ -1249,7 +1249,7 @@
       </c>
       <c r="E8" s="85" t="inlineStr">
         <is>
-          <t>✅ PLATESV-D-2025-001444</t>
+          <t>❓</t>
         </is>
       </c>
     </row>
@@ -1267,7 +1267,7 @@
       </c>
       <c r="E9" s="86" t="inlineStr">
         <is>
-          <t>⚠️ Récente, peu d'historique</t>
+          <t>❓</t>
         </is>
       </c>
     </row>
@@ -1285,7 +1285,7 @@
       </c>
       <c r="E10" s="87" t="inlineStr">
         <is>
-          <t>❓ Non communiquée</t>
+          <t>❓</t>
         </is>
       </c>
     </row>
@@ -1297,7 +1297,7 @@
       </c>
       <c r="E11" s="87" t="inlineStr">
         <is>
-          <t>❓ À vérifier</t>
+          <t>❓</t>
         </is>
       </c>
     </row>
@@ -1314,7 +1314,7 @@
       </c>
       <c r="E12" s="87" t="inlineStr">
         <is>
-          <t>❓ À calculer</t>
+          <t>❓</t>
         </is>
       </c>
     </row>
@@ -1332,7 +1332,7 @@
       </c>
       <c r="E13" s="85" t="inlineStr">
         <is>
-          <t>✅ Professionnel et complet</t>
+          <t>❓</t>
         </is>
       </c>
     </row>
@@ -1350,7 +1350,7 @@
       </c>
       <c r="E14" s="85" t="inlineStr">
         <is>
-          <t>✅ Hist. croissant 300→620 sp.</t>
+          <t>❓</t>
         </is>
       </c>
     </row>
@@ -1368,7 +1368,7 @@
       </c>
       <c r="E15" s="86" t="inlineStr">
         <is>
-          <t>⚠️ NY + Londres à surveiller</t>
+          <t>❓</t>
         </is>
       </c>
     </row>
@@ -1386,7 +1386,7 @@
       </c>
       <c r="E16" s="87" t="inlineStr">
         <is>
-          <t>❓ À calculer</t>
+          <t>❓</t>
         </is>
       </c>
     </row>
@@ -1412,7 +1412,7 @@
       </c>
       <c r="E18" s="88" t="inlineStr">
         <is>
-          <t>Montant</t>
+          <t>❓</t>
         </is>
       </c>
     </row>
@@ -1422,7 +1422,11 @@
           <t>Budget total (éq.)</t>
         </is>
       </c>
-      <c r="E19" s="90" t="n"/>
+      <c r="E19" s="90" t="inlineStr">
+        <is>
+          <t>❓</t>
+        </is>
+      </c>
     </row>
     <row r="20" ht="19.5" customHeight="1" s="77">
       <c r="A20" s="91" t="inlineStr">
@@ -1435,7 +1439,11 @@
           <t>Sub Mairie Paris</t>
         </is>
       </c>
-      <c r="E20" s="90" t="n"/>
+      <c r="E20" s="90" t="inlineStr">
+        <is>
+          <t>❓</t>
+        </is>
+      </c>
     </row>
     <row r="21" ht="13.5" customHeight="1" s="77">
       <c r="A21" s="92" t="inlineStr">
@@ -1449,7 +1457,11 @@
           <t>Dons / partenaires</t>
         </is>
       </c>
-      <c r="E21" s="90" t="n"/>
+      <c r="E21" s="90" t="inlineStr">
+        <is>
+          <t>❓</t>
+        </is>
+      </c>
     </row>
     <row r="22" ht="13.5" customHeight="1" s="77">
       <c r="A22" s="92" t="inlineStr">
@@ -1463,7 +1475,11 @@
           <t>Recettes billetterie</t>
         </is>
       </c>
-      <c r="E22" s="90" t="n"/>
+      <c r="E22" s="90" t="inlineStr">
+        <is>
+          <t>❓</t>
+        </is>
+      </c>
     </row>
     <row r="23" ht="13.5" customHeight="1" s="77">
       <c r="A23" s="92" t="inlineStr">
@@ -1477,7 +1493,11 @@
           <t>Coût moy/jour hors annexes</t>
         </is>
       </c>
-      <c r="E23" s="90" t="n"/>
+      <c r="E23" s="90" t="inlineStr">
+        <is>
+          <t>❓</t>
+        </is>
+      </c>
     </row>
     <row r="24" ht="13.5" customHeight="1" s="77">
       <c r="A24" s="92" t="inlineStr">
@@ -1491,7 +1511,11 @@
           <t>Ratio sub publiques</t>
         </is>
       </c>
-      <c r="E24" s="90" t="n"/>
+      <c r="E24" s="90" t="inlineStr">
+        <is>
+          <t>❓</t>
+        </is>
+      </c>
     </row>
     <row r="25" ht="13.5" customHeight="1" s="77">
       <c r="A25" s="92" t="inlineStr">
@@ -2238,9 +2262,7 @@
           <t>601 Fournitures (trophées, collation, matériel)</t>
         </is>
       </c>
-      <c r="B7" s="112" t="n">
-        <v>910</v>
-      </c>
+      <c r="B7" s="112" t="n"/>
       <c r="D7" s="111" t="inlineStr">
         <is>
           <t>J1 — jauge 150 — prévente (10€) + plein tarif (15€)</t>
@@ -2254,9 +2276,7 @@
           <t>606 Vidéaste &amp; photographe (3 jours)</t>
         </is>
       </c>
-      <c r="B8" s="112" t="n">
-        <v>6200</v>
-      </c>
+      <c r="B8" s="112" t="n"/>
       <c r="D8" s="111" t="inlineStr">
         <is>
           <t>J2 — jauge 150 — prévente + plein tarif</t>
@@ -2317,9 +2337,7 @@
           <t>613 Locations (matériel)</t>
         </is>
       </c>
-      <c r="B12" s="112" t="n">
-        <v>800</v>
-      </c>
+      <c r="B12" s="112" t="n"/>
       <c r="D12" s="110" t="inlineStr">
         <is>
           <t>74 — SUBVENTIONS PUBLIQUES — ⚠️ Toutes à confirmer</t>
@@ -2332,9 +2350,7 @@
           <t>615 Entretien et réparation</t>
         </is>
       </c>
-      <c r="B13" s="112" t="n">
-        <v>400</v>
-      </c>
+      <c r="B13" s="112" t="n"/>
       <c r="D13" s="117" t="inlineStr">
         <is>
           <t>Ville de Paris (AAP HHP26S2) — plafond 10 000€</t>
@@ -2348,9 +2364,7 @@
           <t>616 Assurance</t>
         </is>
       </c>
-      <c r="B14" s="112" t="n">
-        <v>60</v>
-      </c>
+      <c r="B14" s="112" t="n"/>
       <c r="D14" s="117" t="inlineStr">
         <is>
           <t>DRAC Île-de-France</t>
@@ -2408,9 +2422,7 @@
           <t>622 Honoraires coordination générale (Pause Kreyol)</t>
         </is>
       </c>
-      <c r="B18" s="112" t="n">
-        <v>4750</v>
-      </c>
+      <c r="B18" s="112" t="n"/>
       <c r="D18" s="117" t="inlineStr">
         <is>
           <t>Organismes sociaux (CAF, DEETS…)</t>
@@ -2468,9 +2480,7 @@
           <t>623 Publicité et publication</t>
         </is>
       </c>
-      <c r="B22" s="112" t="n">
-        <v>4510</v>
-      </c>
+      <c r="B22" s="112" t="n"/>
       <c r="D22" s="111" t="inlineStr">
         <is>
           <t>Mécénat / fondations privées</t>
@@ -2484,9 +2494,7 @@
           <t>625 VHR déplacements et transports</t>
         </is>
       </c>
-      <c r="B23" s="112" t="n">
-        <v>3200</v>
-      </c>
+      <c r="B23" s="112" t="n"/>
       <c r="D23" s="111" t="inlineStr">
         <is>
           <t>Partenaires culturels privés</t>
@@ -2500,9 +2508,7 @@
           <t>627 Services bancaires</t>
         </is>
       </c>
-      <c r="B24" s="112" t="n">
-        <v>120</v>
-      </c>
+      <c r="B24" s="112" t="n"/>
       <c r="D24" s="111" t="inlineStr">
         <is>
           <t>Dons manuels</t>
@@ -2597,9 +2603,7 @@
           <t>67 Charges exceptionnelles</t>
         </is>
       </c>
-      <c r="B32" s="112" t="n">
-        <v>200</v>
-      </c>
+      <c r="B32" s="112" t="n"/>
     </row>
     <row r="33" ht="12.75" customHeight="1" s="77">
       <c r="A33" s="111" t="inlineStr">
@@ -2607,9 +2611,7 @@
           <t>Charges fixes fonctionnement</t>
         </is>
       </c>
-      <c r="B33" s="112" t="n">
-        <v>1500</v>
-      </c>
+      <c r="B33" s="112" t="n"/>
     </row>
     <row r="34" ht="12.75" customHeight="1" s="77">
       <c r="A34" s="119" t="inlineStr">
@@ -2965,7 +2967,7 @@
       </c>
       <c r="B13" s="133" t="inlineStr">
         <is>
-          <t>300-620 sp. / éd.</t>
+          <t>→ à renseigner</t>
         </is>
       </c>
       <c r="C13" s="130" t="inlineStr">
@@ -2984,6 +2986,7 @@
         </is>
       </c>
     </row>
+    <row r="14"/>
     <row r="15" ht="19.5" customHeight="1" s="77">
       <c r="A15" s="135" t="inlineStr">
         <is>
@@ -2999,7 +3002,7 @@
       </c>
       <c r="B16" s="136" t="inlineStr">
         <is>
-          <t>Niveau</t>
+          <t>→ à renseigner</t>
         </is>
       </c>
       <c r="C16" s="136" t="inlineStr">
@@ -3014,7 +3017,7 @@
       </c>
       <c r="E16" s="136" t="inlineStr">
         <is>
-          <t>Statut</t>
+          <t>❓</t>
         </is>
       </c>
     </row>
@@ -3026,17 +3029,17 @@
       </c>
       <c r="B17" s="137" t="inlineStr">
         <is>
-          <t>MOYEN</t>
+          <t>—</t>
         </is>
       </c>
       <c r="C17" s="138" t="inlineStr">
         <is>
-          <t>Dossiers subventions moins crédibles</t>
+          <t>—</t>
         </is>
       </c>
       <c r="D17" s="139" t="inlineStr">
         <is>
-          <t>Valoriser historique Cie UDP (15 ans)</t>
+          <t>—</t>
         </is>
       </c>
       <c r="E17" s="132" t="inlineStr">
@@ -3053,17 +3056,17 @@
       </c>
       <c r="B18" s="137" t="inlineStr">
         <is>
-          <t>MOYEN</t>
+          <t>—</t>
         </is>
       </c>
       <c r="C18" s="138" t="inlineStr">
         <is>
-          <t>VHR élevés, risque annulation</t>
+          <t>—</t>
         </is>
       </c>
       <c r="D18" s="139" t="inlineStr">
         <is>
-          <t>Contrats signés + assurance annulation</t>
+          <t>—</t>
         </is>
       </c>
       <c r="E18" s="132" t="inlineStr">
@@ -3080,17 +3083,17 @@
       </c>
       <c r="B19" s="140" t="inlineStr">
         <is>
-          <t>ÉLEVÉ</t>
+          <t>—</t>
         </is>
       </c>
       <c r="C19" s="138" t="inlineStr">
         <is>
-          <t>Budget potentiellement non bouclé</t>
+          <t>—</t>
         </is>
       </c>
       <c r="D19" s="139" t="inlineStr">
         <is>
-          <t>Diversifier sources / plan B trésorerie</t>
+          <t>—</t>
         </is>
       </c>
       <c r="E19" s="141" t="inlineStr">
@@ -3107,17 +3110,17 @@
       </c>
       <c r="B20" s="137" t="inlineStr">
         <is>
-          <t>MOYEN</t>
+          <t>—</t>
         </is>
       </c>
       <c r="C20" s="138" t="inlineStr">
         <is>
-          <t>Coût salle non budgété potentiel</t>
+          <t>—</t>
         </is>
       </c>
       <c r="D20" s="139" t="inlineStr">
         <is>
-          <t>Lettre d'engagement avant dépôt dossier</t>
+          <t>—</t>
         </is>
       </c>
       <c r="E20" s="132" t="inlineStr">
@@ -3134,17 +3137,17 @@
       </c>
       <c r="B21" s="142" t="inlineStr">
         <is>
-          <t>FAIBLE</t>
+          <t>—</t>
         </is>
       </c>
       <c r="C21" s="138" t="inlineStr">
         <is>
-          <t>Contentieux potentiel</t>
+          <t>—</t>
         </is>
       </c>
       <c r="D21" s="139" t="inlineStr">
         <is>
-          <t>Contrats de cession systématiques</t>
+          <t>—</t>
         </is>
       </c>
       <c r="E21" s="143" t="inlineStr">
@@ -3161,17 +3164,17 @@
       </c>
       <c r="B22" s="137" t="inlineStr">
         <is>
-          <t>MOYEN</t>
+          <t>—</t>
         </is>
       </c>
       <c r="C22" s="138" t="inlineStr">
         <is>
-          <t>Inéligibilité partielle AAP Mairie</t>
+          <t>—</t>
         </is>
       </c>
       <c r="D22" s="139" t="inlineStr">
         <is>
-          <t>Vérifier ratio dans budget final</t>
+          <t>—</t>
         </is>
       </c>
       <c r="E22" s="132" t="inlineStr">
@@ -3188,17 +3191,17 @@
       </c>
       <c r="B23" s="137" t="inlineStr">
         <is>
-          <t>MOYEN</t>
+          <t>—</t>
         </is>
       </c>
       <c r="C23" s="138" t="inlineStr">
         <is>
-          <t>Incapacité de préfinancement</t>
+          <t>—</t>
         </is>
       </c>
       <c r="D23" s="139" t="inlineStr">
         <is>
-          <t>Demander bilan + situation trésorerie</t>
+          <t>—</t>
         </is>
       </c>
       <c r="E23" s="132" t="inlineStr">
@@ -3215,22 +3218,22 @@
       </c>
       <c r="B24" s="142" t="inlineStr">
         <is>
-          <t>FAIBLE</t>
+          <t>—</t>
         </is>
       </c>
       <c r="C24" s="138" t="inlineStr">
         <is>
-          <t>Recettes inférieures aux prévisions</t>
+          <t>—</t>
         </is>
       </c>
       <c r="D24" s="139" t="inlineStr">
         <is>
-          <t>Historique solide (300→620) rassurant</t>
+          <t>—</t>
         </is>
       </c>
       <c r="E24" s="143" t="inlineStr">
         <is>
-          <t>✅</t>
+          <t>❓</t>
         </is>
       </c>
     </row>
@@ -3399,7 +3402,7 @@
       </c>
       <c r="E32" s="147" t="inlineStr">
         <is>
-          <t>✅</t>
+          <t>☐</t>
         </is>
       </c>
     </row>
@@ -3522,23 +3525,13 @@
       <c r="A39" s="151" t="inlineStr">
         <is>
           <t>✅ POINTS FORTS :
-• 4 éditions avec croissance constante (300 → 620 sp.)
-• Cie UDP : 15 ans d'expérience et réseau solide
-• Licence spectacle obtenue
-• Dossier artistique de qualité professionnelle
-• La Place : partenaire historique et institutionnel
-• Line-up internationale confirmée</t>
+• À compléter après premier entretien</t>
         </is>
       </c>
       <c r="C39" s="152" t="inlineStr">
         <is>
           <t>⚠️ CONDITIONS DE FAISABILITÉ :
-• Confirmation subventions oct 2026 (risque principal)
-• Lettre d'engagement La Place à obtenir d'urgence
-• Bilan comptable asso à fournir (créée sept 2024)
-• Cashets artistes à chiffrer pour budget définitif
-• Vérifier règles 70%/80% aides publiques Mairie
-• Contrats cession droits courts métrages à établir</t>
+• À compléter après analyse</t>
         </is>
       </c>
     </row>
@@ -3548,7 +3541,7 @@
     <row r="43" ht="42" customHeight="1" s="77">
       <c r="A43" s="144" t="inlineStr">
         <is>
-          <t>VERDICT : ✅ PROJET FAISABLE SOUS CONDITIONS — Budget estimé entre 25k€ et 45k€ selon ambition (base éditions précédentes). Faisabilité conditionnée à : (1) confirmation des subventions publiques 2026, (2) lettre d'engagement La Place avant 16 avril, (3) budget artistes définitif avec cachets réels.</t>
+          <t>VERDICT : ❓ À COMPLÉTER — Renseignez les indicateurs ci-dessus</t>
         </is>
       </c>
     </row>

</xml_diff>